<commit_message>
feat: add Excel localization and refine mobile UI with free server plan
</commit_message>
<xml_diff>
--- a/GameData/GameData_MVP.xlsx
+++ b/GameData/GameData_MVP.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="R4388d74f24d147e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdConfig" sheetId="2" r:id="R930c76bb82ff4caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="3" r:id="R1bcfdb05349c465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="R9f0446ee50d74aaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdConfig" sheetId="2" r:id="R8046acef6bd54b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="3" r:id="R67fb549543c6400a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1783,6 +1783,7 @@
     <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="76" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="35" customHeight="1">
@@ -1798,6 +1799,9 @@
       <x:c r="D1" s="5" t="str">
         <x:v>/Description</x:v>
       </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Content_Eng</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="29" customHeight="1">
       <x:c r="A2" s="7" t="str">
@@ -1812,6 +1816,9 @@
       <x:c r="D2" s="7" t="str">
         <x:v>none</x:v>
       </x:c>
+      <x:c r="E2" s="7" t="str">
+        <x:v>string</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="29" customHeight="1">
       <x:c r="A3" s="7" t="str">
@@ -1826,6 +1833,9 @@
       <x:c r="D3" s="7" t="str">
         <x:v>None</x:v>
       </x:c>
+      <x:c r="E3" s="7" t="str">
+        <x:v>Client</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="64" customHeight="1">
       <x:c r="A4" s="8" t="str">
@@ -1840,6 +1850,9 @@
       <x:c r="D4" s="8" t="str">
         <x:v>문구 사용 위치·맥락, 런타임 미출력</x:v>
       </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>영어 표시 문구</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="44" customHeight="1">
       <x:c r="A5" s="16" t="str">
@@ -1854,6 +1867,9 @@
       <x:c r="D5" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E5" s="24" t="str">
+        <x:v>Start with the center</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="44" customHeight="1">
       <x:c r="A6" s="17" t="str">
@@ -1868,6 +1884,9 @@
       <x:c r="D6" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E6" s="25" t="str">
+        <x:v>Connect two stones</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="44" customHeight="1">
       <x:c r="A7" s="16" t="str">
@@ -1882,6 +1901,9 @@
       <x:c r="D7" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>Block the first threat</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="44" customHeight="1">
       <x:c r="A8" s="17" t="str">
@@ -1896,6 +1918,9 @@
       <x:c r="D8" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E8" s="25" t="str">
+        <x:v>Find a horizontal connection</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="44" customHeight="1">
       <x:c r="A9" s="16" t="str">
@@ -1910,6 +1935,9 @@
       <x:c r="D9" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>Take back the center</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="44" customHeight="1">
       <x:c r="A10" s="17" t="str">
@@ -1924,6 +1952,9 @@
       <x:c r="D10" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E10" s="25" t="str">
+        <x:v>Break the AI's connection</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
       <x:c r="A11" s="16" t="str">
@@ -1938,6 +1969,9 @@
       <x:c r="D11" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E11" s="24" t="str">
+        <x:v>Bridge the gap</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="44" customHeight="1">
       <x:c r="A12" s="17" t="str">
@@ -1952,6 +1986,9 @@
       <x:c r="D12" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E12" s="25" t="str">
+        <x:v>Read the AI's opening</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="44" customHeight="1">
       <x:c r="A13" s="16" t="str">
@@ -1966,6 +2003,9 @@
       <x:c r="D13" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E13" s="24" t="str">
+        <x:v>Prepare a fork</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">
       <x:c r="A14" s="17" t="str">
@@ -1980,6 +2020,9 @@
       <x:c r="D14" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E14" s="25" t="str">
+        <x:v>Chapter one review</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="44" customHeight="1">
       <x:c r="A15" s="16" t="str">
@@ -1994,6 +2037,9 @@
       <x:c r="D15" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E15" s="24" t="str">
+        <x:v>Find a diagonal connection</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="44" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -2008,6 +2054,9 @@
       <x:c r="D16" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E16" s="25" t="str">
+        <x:v>Block, then connect</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="44" customHeight="1">
       <x:c r="A17" s="16" t="str">
@@ -2022,6 +2071,9 @@
       <x:c r="D17" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E17" s="24" t="str">
+        <x:v>Choices around the center</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="44" customHeight="1">
       <x:c r="A18" s="17" t="str">
@@ -2036,6 +2088,9 @@
       <x:c r="D18" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E18" s="25" t="str">
+        <x:v>Create two threats</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="44" customHeight="1">
       <x:c r="A19" s="16" t="str">
@@ -2050,6 +2105,9 @@
       <x:c r="D19" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E19" s="24" t="str">
+        <x:v>Find an opening going second</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="44" customHeight="1">
       <x:c r="A20" s="17" t="str">
@@ -2064,6 +2122,9 @@
       <x:c r="D20" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E20" s="25" t="str">
+        <x:v>Block a diagonal threat</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="44" customHeight="1">
       <x:c r="A21" s="16" t="str">
@@ -2078,6 +2139,9 @@
       <x:c r="D21" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E21" s="24" t="str">
+        <x:v>Change direction</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="44" customHeight="1">
       <x:c r="A22" s="17" t="str">
@@ -2092,6 +2156,9 @@
       <x:c r="D22" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E22" s="25" t="str">
+        <x:v>A different kind of fork</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="44" customHeight="1">
       <x:c r="A23" s="16" t="str">
@@ -2106,6 +2173,9 @@
       <x:c r="D23" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E23" s="24" t="str">
+        <x:v>Check the center again</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="44" customHeight="1">
       <x:c r="A24" s="17" t="str">
@@ -2120,6 +2190,9 @@
       <x:c r="D24" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E24" s="25" t="str">
+        <x:v>Review connections and defense</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="44" customHeight="1">
       <x:c r="A25" s="16" t="str">
@@ -2134,6 +2207,9 @@
       <x:c r="D25" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E25" s="24" t="str">
+        <x:v>Connect through a narrow gap</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="44" customHeight="1">
       <x:c r="A26" s="17" t="str">
@@ -2148,6 +2224,9 @@
       <x:c r="D26" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E26" s="25" t="str">
+        <x:v>Defend going second</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="44" customHeight="1">
       <x:c r="A27" s="16" t="str">
@@ -2162,6 +2241,9 @@
       <x:c r="D27" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E27" s="24" t="str">
+        <x:v>The other end of the diagonal</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="44" customHeight="1">
       <x:c r="A28" s="17" t="str">
@@ -2176,6 +2258,9 @@
       <x:c r="D28" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E28" s="25" t="str">
+        <x:v>Compare center and edges</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="44" customHeight="1">
       <x:c r="A29" s="16" t="str">
@@ -2190,6 +2275,9 @@
       <x:c r="D29" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E29" s="24" t="str">
+        <x:v>A complex fork</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="44" customHeight="1">
       <x:c r="A30" s="17" t="str">
@@ -2204,6 +2292,9 @@
       <x:c r="D30" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E30" s="25" t="str">
+        <x:v>Break the AI's diagonal</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="44" customHeight="1">
       <x:c r="A31" s="16" t="str">
@@ -2218,6 +2309,9 @@
       <x:c r="D31" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E31" s="24" t="str">
+        <x:v>Review connections going second</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="44" customHeight="1">
       <x:c r="A32" s="17" t="str">
@@ -2232,6 +2326,9 @@
       <x:c r="D32" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E32" s="25" t="str">
+        <x:v>Find the fork again</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="44" customHeight="1">
       <x:c r="A33" s="16" t="str">
@@ -2246,6 +2343,9 @@
       <x:c r="D33" s="24" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E33" s="24" t="str">
+        <x:v>Final defense practice</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="44" customHeight="1">
       <x:c r="A34" s="17" t="str">
@@ -2260,6 +2360,9 @@
       <x:c r="D34" s="25" t="str">
         <x:v>스테이지 제목</x:v>
       </x:c>
+      <x:c r="E34" s="25" t="str">
+        <x:v>The final tactical challenge</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="44" customHeight="1">
       <x:c r="A35" s="16" t="str">
@@ -2274,6 +2377,9 @@
       <x:c r="D35" s="24" t="str">
         <x:v>내부 작업명, 상점명 미확정</x:v>
       </x:c>
+      <x:c r="E35" s="24" t="str">
+        <x:v>StageGame</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="44" customHeight="1">
       <x:c r="A36" s="17" t="str">
@@ -2288,6 +2394,9 @@
       <x:c r="D36" s="25" t="str">
         <x:v>챕터 1</x:v>
       </x:c>
+      <x:c r="E36" s="25" t="str">
+        <x:v>Center and connections</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="44" customHeight="1">
       <x:c r="A37" s="16" t="str">
@@ -2302,6 +2411,9 @@
       <x:c r="D37" s="24" t="str">
         <x:v>챕터 2</x:v>
       </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>Threats and forks</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="44" customHeight="1">
       <x:c r="A38" s="17" t="str">
@@ -2316,6 +2428,9 @@
       <x:c r="D38" s="25" t="str">
         <x:v>챕터 3</x:v>
       </x:c>
+      <x:c r="E38" s="25" t="str">
+        <x:v>Combined tactics</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="44" customHeight="1">
       <x:c r="A39" s="16" t="str">
@@ -2330,6 +2445,9 @@
       <x:c r="D39" s="24" t="str">
         <x:v>로비 기본 행동</x:v>
       </x:c>
+      <x:c r="E39" s="24" t="str">
+        <x:v>Start</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="44" customHeight="1">
       <x:c r="A40" s="17" t="str">
@@ -2344,6 +2462,9 @@
       <x:c r="D40" s="25" t="str">
         <x:v>최고 해금 스테이지 시작</x:v>
       </x:c>
+      <x:c r="E40" s="25" t="str">
+        <x:v>Continue</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="44" customHeight="1">
       <x:c r="A41" s="16" t="str">
@@ -2358,6 +2479,9 @@
       <x:c r="D41" s="24" t="str">
         <x:v>무료 재도전</x:v>
       </x:c>
+      <x:c r="E41" s="24" t="str">
+        <x:v>Retry</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="44" customHeight="1">
       <x:c r="A42" s="17" t="str">
@@ -2372,6 +2496,9 @@
       <x:c r="D42" s="25" t="str">
         <x:v>승리 후 진행</x:v>
       </x:c>
+      <x:c r="E42" s="25" t="str">
+        <x:v>Next stage</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="44" customHeight="1">
       <x:c r="A43" s="16" t="str">
@@ -2386,6 +2513,9 @@
       <x:c r="D43" s="24" t="str">
         <x:v>결과·설정</x:v>
       </x:c>
+      <x:c r="E43" s="24" t="str">
+        <x:v>Lobby</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="44" customHeight="1">
       <x:c r="A44" s="17" t="str">
@@ -2400,6 +2530,9 @@
       <x:c r="D44" s="25" t="str">
         <x:v>공통 닫기</x:v>
       </x:c>
+      <x:c r="E44" s="25" t="str">
+        <x:v>Close</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="44" customHeight="1">
       <x:c r="A45" s="16" t="str">
@@ -2414,6 +2547,9 @@
       <x:c r="D45" s="24" t="str">
         <x:v>설정 열기</x:v>
       </x:c>
+      <x:c r="E45" s="24" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="44" customHeight="1">
       <x:c r="A46" s="17" t="str">
@@ -2428,6 +2564,9 @@
       <x:c r="D46" s="25" t="str">
         <x:v>규칙 도움말</x:v>
       </x:c>
+      <x:c r="E46" s="25" t="str">
+        <x:v>Help</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="44" customHeight="1">
       <x:c r="A47" s="16" t="str">
@@ -2442,6 +2581,9 @@
       <x:c r="D47" s="24" t="str">
         <x:v>플레이어 턴</x:v>
       </x:c>
+      <x:c r="E47" s="24" t="str">
+        <x:v>Your turn</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="44" customHeight="1">
       <x:c r="A48" s="17" t="str">
@@ -2456,6 +2598,9 @@
       <x:c r="D48" s="25" t="str">
         <x:v>로컬 AI 턴</x:v>
       </x:c>
+      <x:c r="E48" s="25" t="str">
+        <x:v>The AI is thinking</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="44" customHeight="1">
       <x:c r="A49" s="16" t="str">
@@ -2470,6 +2615,9 @@
       <x:c r="D49" s="24" t="str">
         <x:v>플레이어 승리</x:v>
       </x:c>
+      <x:c r="E49" s="24" t="str">
+        <x:v>You win!</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="44" customHeight="1">
       <x:c r="A50" s="17" t="str">
@@ -2484,6 +2632,9 @@
       <x:c r="D50" s="25" t="str">
         <x:v>AI 승리</x:v>
       </x:c>
+      <x:c r="E50" s="25" t="str">
+        <x:v>Try again</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="44" customHeight="1">
       <x:c r="A51" s="16" t="str">
@@ -2498,6 +2649,9 @@
       <x:c r="D51" s="24" t="str">
         <x:v>가득 찬 보드</x:v>
       </x:c>
+      <x:c r="E51" s="24" t="str">
+        <x:v>A draw</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="44" customHeight="1">
       <x:c r="A52" s="17" t="str">
@@ -2512,6 +2666,9 @@
       <x:c r="D52" s="25" t="str">
         <x:v>30스테이지 완료</x:v>
       </x:c>
+      <x:c r="E52" s="25" t="str">
+        <x:v>You have completed all stages</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="44" customHeight="1">
       <x:c r="A53" s="16" t="str">
@@ -2526,6 +2683,9 @@
       <x:c r="D53" s="24" t="str">
         <x:v>규칙</x:v>
       </x:c>
+      <x:c r="E53" s="24" t="str">
+        <x:v>Tap a column to drop a stone. Connect four across, down or diagonally before the AI does.</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="44" customHeight="1">
       <x:c r="A54" s="17" t="str">
@@ -2540,6 +2700,9 @@
       <x:c r="D54" s="25" t="str">
         <x:v>만열 안내</x:v>
       </x:c>
+      <x:c r="E54" s="25" t="str">
+        <x:v>You cannot place a stone in a full column.</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="44" customHeight="1">
       <x:c r="A55" s="16" t="str">
@@ -2554,6 +2717,9 @@
       <x:c r="D55" s="24" t="str">
         <x:v>자발적 리워드 힌트 선택</x:v>
       </x:c>
+      <x:c r="E55" s="24" t="str">
+        <x:v>Watch an ad for a suggested column</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="44" customHeight="1">
       <x:c r="A56" s="17" t="str">
@@ -2568,6 +2734,9 @@
       <x:c r="D56" s="25" t="str">
         <x:v>미충전·실패</x:v>
       </x:c>
+      <x:c r="E56" s="25" t="str">
+        <x:v>No ad is available right now. You can keep playing.</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="44" customHeight="1">
       <x:c r="A57" s="16" t="str">
@@ -2582,6 +2751,9 @@
       <x:c r="D57" s="24" t="str">
         <x:v>보상 최대 1회</x:v>
       </x:c>
+      <x:c r="E57" s="24" t="str">
+        <x:v>You have used this game's ad hint.</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="44" customHeight="1">
       <x:c r="A58" s="17" t="str">
@@ -2596,6 +2768,9 @@
       <x:c r="D58" s="25" t="str">
         <x:v>모의 구현 표기</x:v>
       </x:c>
+      <x:c r="E58" s="25" t="str">
+        <x:v>Ad test mode</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="44" customHeight="1">
       <x:c r="A59" s="16" t="str">
@@ -2610,6 +2785,9 @@
       <x:c r="D59" s="24" t="str">
         <x:v>검증 실패</x:v>
       </x:c>
+      <x:c r="E59" s="24" t="str">
+        <x:v>Game data could not be loaded. Returning to the lobby.</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="44" customHeight="1">
       <x:c r="A60" s="17" t="str">
@@ -2624,6 +2802,9 @@
       <x:c r="D60" s="25" t="str">
         <x:v>저장 실패</x:v>
       </x:c>
+      <x:c r="E60" s="25" t="str">
+        <x:v>Your progress could not be saved.</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="44" customHeight="1">
       <x:c r="A61" s="16" t="str">
@@ -2638,6 +2819,9 @@
       <x:c r="D61" s="24" t="str">
         <x:v>설정</x:v>
       </x:c>
+      <x:c r="E61" s="24" t="str">
+        <x:v>Sound</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="44" customHeight="1">
       <x:c r="A62" s="17" t="str">
@@ -2651,6 +2835,1140 @@
       </x:c>
       <x:c r="D62" s="25" t="str">
         <x:v>설정</x:v>
+      </x:c>
+      <x:c r="E62" s="25" t="str">
+        <x:v>Vibration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="52" customHeight="1">
+      <x:c r="A63" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B63" s="16" t="str">
+        <x:v>client_game_title</x:v>
+      </x:c>
+      <x:c r="C63" s="24" t="str">
+        <x:v>네 개의 수</x:v>
+      </x:c>
+      <x:c r="D63" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E63" s="24" t="str">
+        <x:v>Four in a Row</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="52" customHeight="1">
+      <x:c r="A64" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B64" s="16" t="str">
+        <x:v>game_brand</x:v>
+      </x:c>
+      <x:c r="C64" s="24" t="str">
+        <x:v>STAGEGAME</x:v>
+      </x:c>
+      <x:c r="D64" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E64" s="24" t="str">
+        <x:v>STAGEGAME</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="52" customHeight="1">
+      <x:c r="A65" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B65" s="16" t="str">
+        <x:v>game_subtitle</x:v>
+      </x:c>
+      <x:c r="C65" s="24" t="str">
+        <x:v>한 수씩, 연결되는 전략</x:v>
+      </x:c>
+      <x:c r="D65" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E65" s="24" t="str">
+        <x:v>Connect four. Think ahead.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="52" customHeight="1">
+      <x:c r="A66" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B66" s="16" t="str">
+        <x:v>stage_number</x:v>
+      </x:c>
+      <x:c r="C66" s="24" t="str">
+        <x:v>챕터 {0} · 스테이지 {1}</x:v>
+      </x:c>
+      <x:c r="D66" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E66" s="24" t="str">
+        <x:v>CHAPTER {0} · STAGE {1}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="52" customHeight="1">
+      <x:c r="A67" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B67" s="16" t="str">
+        <x:v>stage_instruction</x:v>
+      </x:c>
+      <x:c r="C67" s="24" t="str">
+        <x:v>가로·세로·대각선으로
+내 돌 4개를 먼저 이으세요.</x:v>
+      </x:c>
+      <x:c r="D67" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E67" s="24" t="str">
+        <x:v>Connect four of your stones
+in any direction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="52" customHeight="1">
+      <x:c r="A68" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B68" s="16" t="str">
+        <x:v>stage_locked_detail</x:v>
+      </x:c>
+      <x:c r="C68" s="24" t="str">
+        <x:v>이전 스테이지에서 승리하면 열립니다.</x:v>
+      </x:c>
+      <x:c r="D68" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E68" s="24" t="str">
+        <x:v>Win the previous stage to unlock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="52" customHeight="1">
+      <x:c r="A69" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B69" s="16" t="str">
+        <x:v>stage_progress</x:v>
+      </x:c>
+      <x:c r="C69" s="24" t="str">
+        <x:v>{0} / {1} 스테이지 해금</x:v>
+      </x:c>
+      <x:c r="D69" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E69" s="24" t="str">
+        <x:v>{0} / {1} stages unlocked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="52" customHeight="1">
+      <x:c r="A70" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B70" s="16" t="str">
+        <x:v>client_ui_start</x:v>
+      </x:c>
+      <x:c r="C70" s="24" t="str">
+        <x:v>대국 시작</x:v>
+      </x:c>
+      <x:c r="D70" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E70" s="24" t="str">
+        <x:v>Play</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="52" customHeight="1">
+      <x:c r="A71" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B71" s="16" t="str">
+        <x:v>stage_locked</x:v>
+      </x:c>
+      <x:c r="C71" s="24" t="str">
+        <x:v>잠긴 스테이지</x:v>
+      </x:c>
+      <x:c r="D71" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E71" s="24" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="52" customHeight="1">
+      <x:c r="A72" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B72" s="16" t="str">
+        <x:v>ui_previous_page</x:v>
+      </x:c>
+      <x:c r="C72" s="24" t="str">
+        <x:v>이전</x:v>
+      </x:c>
+      <x:c r="D72" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E72" s="24" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="52" customHeight="1">
+      <x:c r="A73" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B73" s="16" t="str">
+        <x:v>ui_next_page</x:v>
+      </x:c>
+      <x:c r="C73" s="24" t="str">
+        <x:v>다음</x:v>
+      </x:c>
+      <x:c r="D73" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E73" s="24" t="str">
+        <x:v>Next</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="52" customHeight="1">
+      <x:c r="A74" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B74" s="16" t="str">
+        <x:v>client_ui_help</x:v>
+      </x:c>
+      <x:c r="C74" s="24" t="str">
+        <x:v>플레이 방법</x:v>
+      </x:c>
+      <x:c r="D74" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E74" s="24" t="str">
+        <x:v>How to play</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="52" customHeight="1">
+      <x:c r="A75" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B75" s="16" t="str">
+        <x:v>lobby_notice</x:v>
+      </x:c>
+      <x:c r="C75" s="24" t="str">
+        <x:v>진행도는 이 기기에 저장됩니다</x:v>
+      </x:c>
+      <x:c r="D75" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E75" s="24" t="str">
+        <x:v>Progress is saved on this device</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="52" customHeight="1">
+      <x:c r="A76" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B76" s="16" t="str">
+        <x:v>match_eyebrow</x:v>
+      </x:c>
+      <x:c r="C76" s="24" t="str">
+        <x:v>4목 대국</x:v>
+      </x:c>
+      <x:c r="D76" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E76" s="24" t="str">
+        <x:v>FOUR IN A ROW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="52" customHeight="1">
+      <x:c r="A77" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B77" s="16" t="str">
+        <x:v>match_title</x:v>
+      </x:c>
+      <x:c r="C77" s="24" t="str">
+        <x:v>{0} · {1}</x:v>
+      </x:c>
+      <x:c r="D77" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E77" s="24" t="str">
+        <x:v>{0} · {1}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="52" customHeight="1">
+      <x:c r="A78" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B78" s="16" t="str">
+        <x:v>ui_pause</x:v>
+      </x:c>
+      <x:c r="C78" s="24" t="str">
+        <x:v>쉼</x:v>
+      </x:c>
+      <x:c r="D78" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E78" s="24" t="str">
+        <x:v>Pause</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="52" customHeight="1">
+      <x:c r="A79" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B79" s="16" t="str">
+        <x:v>match_legend</x:v>
+      </x:c>
+      <x:c r="C79" s="24" t="str">
+        <x:v>나 · 민트   /   AI · 산호</x:v>
+      </x:c>
+      <x:c r="D79" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E79" s="24" t="str">
+        <x:v>You · Mint   /   AI · Coral</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="52" customHeight="1">
+      <x:c r="A80" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B80" s="16" t="str">
+        <x:v>match_instruction</x:v>
+      </x:c>
+      <x:c r="C80" s="24" t="str">
+        <x:v>돌을 놓을 열을 선택하세요.</x:v>
+      </x:c>
+      <x:c r="D80" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E80" s="24" t="str">
+        <x:v>Choose a column to drop a stone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="52" customHeight="1">
+      <x:c r="A81" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B81" s="16" t="str">
+        <x:v>player_stone</x:v>
+      </x:c>
+      <x:c r="C81" s="24" t="str">
+        <x:v>나</x:v>
+      </x:c>
+      <x:c r="D81" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E81" s="24" t="str">
+        <x:v>You</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="52" customHeight="1">
+      <x:c r="A82" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B82" s="16" t="str">
+        <x:v>ai_stone</x:v>
+      </x:c>
+      <x:c r="C82" s="24" t="str">
+        <x:v>AI</x:v>
+      </x:c>
+      <x:c r="D82" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E82" s="24" t="str">
+        <x:v>AI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="52" customHeight="1">
+      <x:c r="A83" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B83" s="16" t="str">
+        <x:v>column_number</x:v>
+      </x:c>
+      <x:c r="C83" s="24" t="str">
+        <x:v>{0}</x:v>
+      </x:c>
+      <x:c r="D83" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E83" s="24" t="str">
+        <x:v>{0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="52" customHeight="1">
+      <x:c r="A84" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B84" s="16" t="str">
+        <x:v>move_count</x:v>
+      </x:c>
+      <x:c r="C84" s="24" t="str">
+        <x:v>{0} / 42 수</x:v>
+      </x:c>
+      <x:c r="D84" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E84" s="24" t="str">
+        <x:v>{0} / 42 moves</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="52" customHeight="1">
+      <x:c r="A85" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B85" s="16" t="str">
+        <x:v>turn_finished</x:v>
+      </x:c>
+      <x:c r="C85" s="24" t="str">
+        <x:v>대국 종료</x:v>
+      </x:c>
+      <x:c r="D85" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E85" s="24" t="str">
+        <x:v>Game over</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="52" customHeight="1">
+      <x:c r="A86" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B86" s="16" t="str">
+        <x:v>turn_thinking</x:v>
+      </x:c>
+      <x:c r="C86" s="24" t="str">
+        <x:v>다음 수를 살펴보는 중…</x:v>
+      </x:c>
+      <x:c r="D86" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E86" s="24" t="str">
+        <x:v>Thinking…</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="52" customHeight="1">
+      <x:c r="A87" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B87" s="16" t="str">
+        <x:v>client_ui_player_turn</x:v>
+      </x:c>
+      <x:c r="C87" s="24" t="str">
+        <x:v>내 차례 · 열을 선택하세요</x:v>
+      </x:c>
+      <x:c r="D87" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E87" s="24" t="str">
+        <x:v>Your turn · Choose a column</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="52" customHeight="1">
+      <x:c r="A88" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B88" s="16" t="str">
+        <x:v>client_ui_ai_turn</x:v>
+      </x:c>
+      <x:c r="C88" s="24" t="str">
+        <x:v>AI 차례</x:v>
+      </x:c>
+      <x:c r="D88" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E88" s="24" t="str">
+        <x:v>AI's turn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="52" customHeight="1">
+      <x:c r="A89" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B89" s="16" t="str">
+        <x:v>client_hint_request</x:v>
+      </x:c>
+      <x:c r="C89" s="24" t="str">
+        <x:v>광고 보고 힌트 · 1회</x:v>
+      </x:c>
+      <x:c r="D89" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E89" s="24" t="str">
+        <x:v>Watch ad for hint · Once</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="52" customHeight="1">
+      <x:c r="A90" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B90" s="16" t="str">
+        <x:v>client_hint_unavailable</x:v>
+      </x:c>
+      <x:c r="C90" s="24" t="str">
+        <x:v>광고가 준비되지 않았어요. 계속 플레이하세요.</x:v>
+      </x:c>
+      <x:c r="D90" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E90" s="24" t="str">
+        <x:v>No ad available. Keep playing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="52" customHeight="1">
+      <x:c r="A91" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B91" s="16" t="str">
+        <x:v>hint_incomplete</x:v>
+      </x:c>
+      <x:c r="C91" s="24" t="str">
+        <x:v>광고가 완료되지 않아 힌트를 받지 못했어요.</x:v>
+      </x:c>
+      <x:c r="D91" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E91" s="24" t="str">
+        <x:v>Ad not completed. No hint used.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="52" customHeight="1">
+      <x:c r="A92" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B92" s="16" t="str">
+        <x:v>hint_timeout</x:v>
+      </x:c>
+      <x:c r="C92" s="24" t="str">
+        <x:v>광고 응답이 없어 취소했어요. 계속 플레이하세요.</x:v>
+      </x:c>
+      <x:c r="D92" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E92" s="24" t="str">
+        <x:v>Ad timed out. Keep playing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="52" customHeight="1">
+      <x:c r="A93" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B93" s="16" t="str">
+        <x:v>hint_cancelled</x:v>
+      </x:c>
+      <x:c r="C93" s="24" t="str">
+        <x:v>광고 요청을 취소했어요. 계속 플레이하세요.</x:v>
+      </x:c>
+      <x:c r="D93" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E93" s="24" t="str">
+        <x:v>Ad cancelled. Keep playing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="52" customHeight="1">
+      <x:c r="A94" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B94" s="16" t="str">
+        <x:v>hint_recommendation</x:v>
+      </x:c>
+      <x:c r="C94" s="24" t="str">
+        <x:v>추천: {0}번 열</x:v>
+      </x:c>
+      <x:c r="D94" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E94" s="24" t="str">
+        <x:v>Try column {0}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="52" customHeight="1">
+      <x:c r="A95" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B95" s="16" t="str">
+        <x:v>client_hint_used</x:v>
+      </x:c>
+      <x:c r="C95" s="24" t="str">
+        <x:v>이번 판 힌트 사용 완료</x:v>
+      </x:c>
+      <x:c r="D95" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E95" s="24" t="str">
+        <x:v>Hint used this game</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="52" customHeight="1">
+      <x:c r="A96" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B96" s="16" t="str">
+        <x:v>client_result_win</x:v>
+      </x:c>
+      <x:c r="C96" s="24" t="str">
+        <x:v>연결 성공!</x:v>
+      </x:c>
+      <x:c r="D96" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E96" s="24" t="str">
+        <x:v>Four connected!</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="52" customHeight="1">
+      <x:c r="A97" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B97" s="16" t="str">
+        <x:v>client_result_loss</x:v>
+      </x:c>
+      <x:c r="C97" s="24" t="str">
+        <x:v>다시 도전해 볼까요?</x:v>
+      </x:c>
+      <x:c r="D97" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E97" s="24" t="str">
+        <x:v>Try again?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="52" customHeight="1">
+      <x:c r="A98" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B98" s="16" t="str">
+        <x:v>result_win_detail</x:v>
+      </x:c>
+      <x:c r="C98" s="24" t="str">
+        <x:v>네 개의 돌을 이었어요.
+다음 스테이지에 도전하세요.</x:v>
+      </x:c>
+      <x:c r="D98" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E98" s="24" t="str">
+        <x:v>You connected four stones.
+Try the next stage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="52" customHeight="1">
+      <x:c r="A99" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B99" s="16" t="str">
+        <x:v>result_draw_detail</x:v>
+      </x:c>
+      <x:c r="C99" s="24" t="str">
+        <x:v>42칸이 모두 찼어요.
+다시 도전해 보세요.</x:v>
+      </x:c>
+      <x:c r="D99" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E99" s="24" t="str">
+        <x:v>All 42 spaces are full.
+Give it another try.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="52" customHeight="1">
+      <x:c r="A100" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B100" s="16" t="str">
+        <x:v>result_loss_detail</x:v>
+      </x:c>
+      <x:c r="C100" s="24" t="str">
+        <x:v>상대가 먼저 네 개를 이었어요.
+다음에는 세 돌 연결을 막아 보세요.</x:v>
+      </x:c>
+      <x:c r="D100" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E100" s="24" t="str">
+        <x:v>The AI connected four first.
+Watch for lines of three.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="52" customHeight="1">
+      <x:c r="A101" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B101" s="16" t="str">
+        <x:v>result_loss_horizontal</x:v>
+      </x:c>
+      <x:c r="C101" s="24" t="str">
+        <x:v>AI가 가로로 네 개를 이었어요.
+금색 줄을 살펴보세요.</x:v>
+      </x:c>
+      <x:c r="D101" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E101" s="24" t="str">
+        <x:v>The AI connected four across.
+Look at the gold line.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="52" customHeight="1">
+      <x:c r="A102" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B102" s="16" t="str">
+        <x:v>result_loss_vertical</x:v>
+      </x:c>
+      <x:c r="C102" s="24" t="str">
+        <x:v>AI가 세로로 네 개를 이었어요.
+금색 줄을 살펴보세요.</x:v>
+      </x:c>
+      <x:c r="D102" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E102" s="24" t="str">
+        <x:v>The AI connected four vertically.
+Look at the gold line.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="52" customHeight="1">
+      <x:c r="A103" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B103" s="16" t="str">
+        <x:v>result_loss_diagonal</x:v>
+      </x:c>
+      <x:c r="C103" s="24" t="str">
+        <x:v>AI가 대각선으로 네 개를 이었어요.
+금색 줄을 살펴보세요.</x:v>
+      </x:c>
+      <x:c r="D103" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E103" s="24" t="str">
+        <x:v>The AI connected four diagonally.
+Look at the gold line.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="52" customHeight="1">
+      <x:c r="A104" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B104" s="16" t="str">
+        <x:v>client_result_all_clear</x:v>
+      </x:c>
+      <x:c r="C104" s="24" t="str">
+        <x:v>모든 스테이지 완료!
+원하는 스테이지를 다시 즐겨 보세요.</x:v>
+      </x:c>
+      <x:c r="D104" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E104" s="24" t="str">
+        <x:v>All stages complete!
+Replay any stage you like.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="52" customHeight="1">
+      <x:c r="A105" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B105" s="16" t="str">
+        <x:v>client_ui_continue</x:v>
+      </x:c>
+      <x:c r="C105" s="24" t="str">
+        <x:v>이어서 대국</x:v>
+      </x:c>
+      <x:c r="D105" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E105" s="24" t="str">
+        <x:v>Resume</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="52" customHeight="1">
+      <x:c r="A106" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B106" s="16" t="str">
+        <x:v>confirm_title</x:v>
+      </x:c>
+      <x:c r="C106" s="24" t="str">
+        <x:v>잠시 쉬어가기</x:v>
+      </x:c>
+      <x:c r="D106" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E106" s="24" t="str">
+        <x:v>Paused</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="52" customHeight="1">
+      <x:c r="A107" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B107" s="16" t="str">
+        <x:v>confirm_body</x:v>
+      </x:c>
+      <x:c r="C107" s="24" t="str">
+        <x:v>현재 대국은 저장되지 않아요.
+해금한 스테이지는 유지됩니다.</x:v>
+      </x:c>
+      <x:c r="D107" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E107" s="24" t="str">
+        <x:v>This game won't be saved.
+Unlocked stages stay available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="52" customHeight="1">
+      <x:c r="A108" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B108" s="16" t="str">
+        <x:v>confirm_leave</x:v>
+      </x:c>
+      <x:c r="C108" s="24" t="str">
+        <x:v>로비로 나가기</x:v>
+      </x:c>
+      <x:c r="D108" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E108" s="24" t="str">
+        <x:v>Leave game</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="52" customHeight="1">
+      <x:c r="A109" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B109" s="16" t="str">
+        <x:v>settings_detail</x:v>
+      </x:c>
+      <x:c r="C109" s="24" t="str">
+        <x:v>진행도는 이 기기에 저장됩니다.</x:v>
+      </x:c>
+      <x:c r="D109" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E109" s="24" t="str">
+        <x:v>Progress is saved on this device.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="52" customHeight="1">
+      <x:c r="A110" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B110" s="16" t="str">
+        <x:v>settings_sound_on</x:v>
+      </x:c>
+      <x:c r="C110" s="24" t="str">
+        <x:v>효과음 켜짐</x:v>
+      </x:c>
+      <x:c r="D110" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E110" s="24" t="str">
+        <x:v>Sound on</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="52" customHeight="1">
+      <x:c r="A111" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B111" s="16" t="str">
+        <x:v>settings_sound_off</x:v>
+      </x:c>
+      <x:c r="C111" s="24" t="str">
+        <x:v>효과음 꺼짐</x:v>
+      </x:c>
+      <x:c r="D111" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E111" s="24" t="str">
+        <x:v>Sound off</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="52" customHeight="1">
+      <x:c r="A112" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B112" s="16" t="str">
+        <x:v>settings_language</x:v>
+      </x:c>
+      <x:c r="C112" s="24" t="str">
+        <x:v>언어 / Language</x:v>
+      </x:c>
+      <x:c r="D112" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E112" s="24" t="str">
+        <x:v>언어 / Language</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="52" customHeight="1">
+      <x:c r="A113" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B113" s="16" t="str">
+        <x:v>language_ko</x:v>
+      </x:c>
+      <x:c r="C113" s="24" t="str">
+        <x:v>한국어</x:v>
+      </x:c>
+      <x:c r="D113" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E113" s="24" t="str">
+        <x:v>한국어</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="52" customHeight="1">
+      <x:c r="A114" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B114" s="16" t="str">
+        <x:v>language_en</x:v>
+      </x:c>
+      <x:c r="C114" s="24" t="str">
+        <x:v>English</x:v>
+      </x:c>
+      <x:c r="D114" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E114" s="24" t="str">
+        <x:v>English</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="52" customHeight="1">
+      <x:c r="A115" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B115" s="16" t="str">
+        <x:v>language_selected</x:v>
+      </x:c>
+      <x:c r="C115" s="24" t="str">
+        <x:v>{0} ✓</x:v>
+      </x:c>
+      <x:c r="D115" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E115" s="24" t="str">
+        <x:v>{0} ✓</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="52" customHeight="1">
+      <x:c r="A116" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B116" s="16" t="str">
+        <x:v>legal_title</x:v>
+      </x:c>
+      <x:c r="C116" s="24" t="str">
+        <x:v>오픈소스 라이선스</x:v>
+      </x:c>
+      <x:c r="D116" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E116" s="24" t="str">
+        <x:v>Open source licenses</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="52" customHeight="1">
+      <x:c r="A117" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B117" s="16" t="str">
+        <x:v>legal_missing</x:v>
+      </x:c>
+      <x:c r="C117" s="24" t="str">
+        <x:v>라이선스 파일을 불러올 수 없어요.</x:v>
+      </x:c>
+      <x:c r="D117" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E117" s="24" t="str">
+        <x:v>Licenses could not be loaded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="152" customHeight="1">
+      <x:c r="A118" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B118" s="16" t="str">
+        <x:v>client_help_rules</x:v>
+      </x:c>
+      <x:c r="C118" s="24" t="str">
+        <x:v>1. 열을 누르면 돌이 아래로 떨어져요.
+2. 가로·세로·대각선으로 네 개를 이으세요.
+3. 상대의 세 돌 연결을 먼저 막으세요.
+금색 줄은 승리한 연결이에요.</x:v>
+      </x:c>
+      <x:c r="D118" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E118" s="24" t="str">
+        <x:v>1. Tap a column to drop a stone.
+2. Connect four across, down or diagonally.
+3. Block the AI's lines of three.
+The winning line turns gold.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="52" customHeight="1">
+      <x:c r="A119" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B119" s="16" t="str">
+        <x:v>ad_unavailable</x:v>
+      </x:c>
+      <x:c r="C119" s="24" t="str">
+        <x:v>광고를 준비하지 못했어요.</x:v>
+      </x:c>
+      <x:c r="D119" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E119" s="24" t="str">
+        <x:v>No ad available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="52" customHeight="1">
+      <x:c r="A120" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B120" s="16" t="str">
+        <x:v>client_ad_test_mode</x:v>
+      </x:c>
+      <x:c r="C120" s="24" t="str">
+        <x:v>모의 광고 · 테스트 전용</x:v>
+      </x:c>
+      <x:c r="D120" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E120" s="24" t="str">
+        <x:v>Mock ad · Test only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="52" customHeight="1">
+      <x:c r="A121" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B121" s="16" t="str">
+        <x:v>error_data_title</x:v>
+      </x:c>
+      <x:c r="C121" s="24" t="str">
+        <x:v>데이터 확인 필요</x:v>
+      </x:c>
+      <x:c r="D121" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E121" s="24" t="str">
+        <x:v>Data unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="52" customHeight="1">
+      <x:c r="A122" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B122" s="16" t="str">
+        <x:v>client_error_data</x:v>
+      </x:c>
+      <x:c r="C122" s="24" t="str">
+        <x:v>게임을 불러올 수 없어요.
+다시 실행해 주세요.</x:v>
+      </x:c>
+      <x:c r="D122" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E122" s="24" t="str">
+        <x:v>The game could not load.
+Please restart.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="52" customHeight="1">
+      <x:c r="A123" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B123" s="16" t="str">
+        <x:v>client_error_save</x:v>
+      </x:c>
+      <x:c r="C123" s="24" t="str">
+        <x:v>저장하지 못했어요. 재실행하면 진행도가 사라질 수 있어요.</x:v>
+      </x:c>
+      <x:c r="D123" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E123" s="24" t="str">
+        <x:v>Could not save. Progress may be lost after restart.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="52" customHeight="1">
+      <x:c r="A124" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B124" s="16" t="str">
+        <x:v>error_load</x:v>
+      </x:c>
+      <x:c r="C124" s="24" t="str">
+        <x:v>저장을 복원하지 못해 처음부터 시작해요.</x:v>
+      </x:c>
+      <x:c r="D124" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E124" s="24" t="str">
+        <x:v>Save could not be restored. Starting over.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="52" customHeight="1">
+      <x:c r="A125" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B125" s="16" t="str">
+        <x:v>web_loading</x:v>
+      </x:c>
+      <x:c r="C125" s="24" t="str">
+        <x:v>게임을 불러오는 중…</x:v>
+      </x:c>
+      <x:c r="D125" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E125" s="24" t="str">
+        <x:v>Loading game…</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="52" customHeight="1">
+      <x:c r="A126" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B126" s="16" t="str">
+        <x:v>web_error</x:v>
+      </x:c>
+      <x:c r="C126" s="24" t="str">
+        <x:v>게임을 불러올 수 없어요. 새로고침해 주세요.</x:v>
+      </x:c>
+      <x:c r="D126" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E126" s="24" t="str">
+        <x:v>Could not load the game. Please reload.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="52" customHeight="1">
+      <x:c r="A127" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B127" s="16" t="str">
+        <x:v>web_canvas_label</x:v>
+      </x:c>
+      <x:c r="C127" s="24" t="str">
+        <x:v>네 개의 수 게임</x:v>
+      </x:c>
+      <x:c r="D127" s="24" t="str">
+        <x:v>UI 언어 전환</x:v>
+      </x:c>
+      <x:c r="E127" s="24" t="str">
+        <x:v>Four in a Row game</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: clarify stage progression and illustrated rules
</commit_message>
<xml_diff>
--- a/GameData/GameData_MVP.xlsx
+++ b/GameData/GameData_MVP.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="R9f0446ee50d74aaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdConfig" sheetId="2" r:id="R8046acef6bd54b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="3" r:id="R67fb549543c6400a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" r:id="R8dfcdef817144db2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdConfig" sheetId="2" r:id="Rf13af8dea2a04837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strings" sheetId="3" r:id="R6fbc666b133a42b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3502,15 +3502,13 @@
         <x:v>result_loss_horizontal</x:v>
       </x:c>
       <x:c r="C101" s="24" t="str">
-        <x:v>AI가 가로로 네 개를 이었어요.
-금색 줄을 살펴보세요.</x:v>
+        <x:v>AI가 가로로 네 개를 이었어요.</x:v>
       </x:c>
       <x:c r="D101" s="24" t="str">
         <x:v>UI 언어 전환</x:v>
       </x:c>
       <x:c r="E101" s="24" t="str">
-        <x:v>The AI connected four across.
-Look at the gold line.</x:v>
+        <x:v>The AI connected four across.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="52" customHeight="1">
@@ -3521,15 +3519,13 @@
         <x:v>result_loss_vertical</x:v>
       </x:c>
       <x:c r="C102" s="24" t="str">
-        <x:v>AI가 세로로 네 개를 이었어요.
-금색 줄을 살펴보세요.</x:v>
+        <x:v>AI가 세로로 네 개를 이었어요.</x:v>
       </x:c>
       <x:c r="D102" s="24" t="str">
         <x:v>UI 언어 전환</x:v>
       </x:c>
       <x:c r="E102" s="24" t="str">
-        <x:v>The AI connected four vertically.
-Look at the gold line.</x:v>
+        <x:v>The AI connected four vertically.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="52" customHeight="1">
@@ -3540,15 +3536,13 @@
         <x:v>result_loss_diagonal</x:v>
       </x:c>
       <x:c r="C103" s="24" t="str">
-        <x:v>AI가 대각선으로 네 개를 이었어요.
-금색 줄을 살펴보세요.</x:v>
+        <x:v>AI가 대각선으로 네 개를 이었어요.</x:v>
       </x:c>
       <x:c r="D103" s="24" t="str">
         <x:v>UI 언어 전환</x:v>
       </x:c>
       <x:c r="E103" s="24" t="str">
-        <x:v>The AI connected four diagonally.
-Look at the gold line.</x:v>
+        <x:v>The AI connected four diagonally.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="52" customHeight="1">
@@ -3969,6 +3963,244 @@
       </x:c>
       <x:c r="E127" s="24" t="str">
         <x:v>Four in a Row game</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="52" customHeight="1">
+      <x:c r="A128" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B128" s="16" t="str">
+        <x:v>stage_map_chapter</x:v>
+      </x:c>
+      <x:c r="C128" s="24" t="str">
+        <x:v>{0} / {1} 챕터</x:v>
+      </x:c>
+      <x:c r="D128" s="24" t="str">
+        <x:v>단계 선택 챕터 번호</x:v>
+      </x:c>
+      <x:c r="E128" s="24" t="str">
+        <x:v>Chapter {0} / {1}</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="52" customHeight="1">
+      <x:c r="A129" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B129" s="16" t="str">
+        <x:v>stage_tier_1</x:v>
+      </x:c>
+      <x:c r="C129" s="24" t="str">
+        <x:v>입문</x:v>
+      </x:c>
+      <x:c r="D129" s="24" t="str">
+        <x:v>1–10 챕터 표시명, 실제 난이도 검증 아님</x:v>
+      </x:c>
+      <x:c r="E129" s="24" t="str">
+        <x:v>Basics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="52" customHeight="1">
+      <x:c r="A130" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B130" s="16" t="str">
+        <x:v>stage_tier_2</x:v>
+      </x:c>
+      <x:c r="C130" s="24" t="str">
+        <x:v>전술</x:v>
+      </x:c>
+      <x:c r="D130" s="24" t="str">
+        <x:v>11–20 챕터 표시명, 실제 난이도 검증 아님</x:v>
+      </x:c>
+      <x:c r="E130" s="24" t="str">
+        <x:v>Tactics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="52" customHeight="1">
+      <x:c r="A131" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B131" s="16" t="str">
+        <x:v>stage_tier_3</x:v>
+      </x:c>
+      <x:c r="C131" s="24" t="str">
+        <x:v>도전</x:v>
+      </x:c>
+      <x:c r="D131" s="24" t="str">
+        <x:v>21–30 챕터 표시명, 실제 난이도 검증 아님</x:v>
+      </x:c>
+      <x:c r="E131" s="24" t="str">
+        <x:v>Challenge</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="52" customHeight="1">
+      <x:c r="A132" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B132" s="16" t="str">
+        <x:v>stage_state_cleared</x:v>
+      </x:c>
+      <x:c r="C132" s="24" t="str">
+        <x:v>완료</x:v>
+      </x:c>
+      <x:c r="D132" s="24" t="str">
+        <x:v>단계 완료 상태</x:v>
+      </x:c>
+      <x:c r="E132" s="24" t="str">
+        <x:v>Clear</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="52" customHeight="1">
+      <x:c r="A133" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B133" s="16" t="str">
+        <x:v>stage_state_current</x:v>
+      </x:c>
+      <x:c r="C133" s="24" t="str">
+        <x:v>도전</x:v>
+      </x:c>
+      <x:c r="D133" s="24" t="str">
+        <x:v>현재 도전 단계 상태</x:v>
+      </x:c>
+      <x:c r="E133" s="24" t="str">
+        <x:v>Play</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="52" customHeight="1">
+      <x:c r="A134" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B134" s="16" t="str">
+        <x:v>stage_state_locked</x:v>
+      </x:c>
+      <x:c r="C134" s="24" t="str">
+        <x:v>잠금</x:v>
+      </x:c>
+      <x:c r="D134" s="24" t="str">
+        <x:v>미해금 단계 상태</x:v>
+      </x:c>
+      <x:c r="E134" s="24" t="str">
+        <x:v>Locked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="52" customHeight="1">
+      <x:c r="A135" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B135" s="16" t="str">
+        <x:v>stage_cleared_progress</x:v>
+      </x:c>
+      <x:c r="C135" s="24" t="str">
+        <x:v>{0}/{1} 완료</x:v>
+      </x:c>
+      <x:c r="D135" s="24" t="str">
+        <x:v>완료 단계 수와 전체 단계 수</x:v>
+      </x:c>
+      <x:c r="E135" s="24" t="str">
+        <x:v>{0}/{1} cleared</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="52" customHeight="1">
+      <x:c r="A136" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B136" s="16" t="str">
+        <x:v>stage_replay</x:v>
+      </x:c>
+      <x:c r="C136" s="24" t="str">
+        <x:v>다시 도전</x:v>
+      </x:c>
+      <x:c r="D136" s="24" t="str">
+        <x:v>완료 단계 다시 도전</x:v>
+      </x:c>
+      <x:c r="E136" s="24" t="str">
+        <x:v>Play again</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="52" customHeight="1">
+      <x:c r="A137" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B137" s="16" t="str">
+        <x:v>stage_lock_requirement</x:v>
+      </x:c>
+      <x:c r="C137" s="24" t="str">
+        <x:v>{0} 스테이지를 먼저 완료하세요</x:v>
+      </x:c>
+      <x:c r="D137" s="24" t="str">
+        <x:v>잠금 해제 선행 단계 안내</x:v>
+      </x:c>
+      <x:c r="E137" s="24" t="str">
+        <x:v>Clear stage {0} first</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="52" customHeight="1">
+      <x:c r="A138" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B138" s="16" t="str">
+        <x:v>help_drop_title</x:v>
+      </x:c>
+      <x:c r="C138" s="24" t="str">
+        <x:v>열을 고르면 아래로</x:v>
+      </x:c>
+      <x:c r="D138" s="24" t="str">
+        <x:v>그림 도움말 제목: 돌 놓기</x:v>
+      </x:c>
+      <x:c r="E138" s="24" t="str">
+        <x:v>Choose a column</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="52" customHeight="1">
+      <x:c r="A139" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B139" s="16" t="str">
+        <x:v>help_drop_caption</x:v>
+      </x:c>
+      <x:c r="C139" s="24" t="str">
+        <x:v>돌은 가장 아래 빈칸에 놓여요</x:v>
+      </x:c>
+      <x:c r="D139" s="24" t="str">
+        <x:v>그림 도움말 설명: 돌 놓기</x:v>
+      </x:c>
+      <x:c r="E139" s="24" t="str">
+        <x:v>Your stone falls into the lowest empty space</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="52" customHeight="1">
+      <x:c r="A140" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B140" s="16" t="str">
+        <x:v>help_connect_title</x:v>
+      </x:c>
+      <x:c r="C140" s="24" t="str">
+        <x:v>네 개를 연결하면 승리</x:v>
+      </x:c>
+      <x:c r="D140" s="24" t="str">
+        <x:v>그림 도움말 제목: 승리 조건</x:v>
+      </x:c>
+      <x:c r="E140" s="24" t="str">
+        <x:v>Connect four to win</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="52" customHeight="1">
+      <x:c r="A141" s="16" t="str">
+        <x:v>USE</x:v>
+      </x:c>
+      <x:c r="B141" s="16" t="str">
+        <x:v>help_connect_caption</x:v>
+      </x:c>
+      <x:c r="C141" s="24" t="str">
+        <x:v>가로 · 세로 · 대각선</x:v>
+      </x:c>
+      <x:c r="D141" s="24" t="str">
+        <x:v>그림 도움말 설명: 연결 방향</x:v>
+      </x:c>
+      <x:c r="E141" s="24" t="str">
+        <x:v>Across · Up · Diagonal</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>